<commit_message>
docs(testes): adiciona avaliacao heuristica do GuiaCidadao (PDF e planilha)
Relatorio individual de avaliacao heuristica (Laise) com 5 problemas reais
identificados no app em execucao e suas evidencias, alem da planilha
consolidada por heuristica. Entrega final em PDF; versao DOCX removida.

Correcoes de usabilidade aplicadas a partir dos achados:
- Painel do Colaborador: acentuacao de "Olá" e "Acesso rápido".
- Sessao local: remove o hash de senha do objeto gravado em localStorage (LGPD).
</commit_message>
<xml_diff>
--- a/docs/testes/avaliacao-heuristica/Avaliacao_Heuristica_Consolidada.xlsx
+++ b/docs/testes/avaliacao-heuristica/Avaliacao_Heuristica_Consolidada.xlsx
@@ -1,12 +1,12 @@
 
 <file path=xl/workbook.xml><?xml version="1.0" encoding="utf-8"?>
-<workbook xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
+<workbook xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main">
   <workbookPr/>
   <bookViews>
     <workbookView visibility="visible" minimized="0" showHorizontalScroll="1" showVerticalScroll="1" showSheetTabs="1" xWindow="0" yWindow="0" windowWidth="16380" windowHeight="8196" tabRatio="500" firstSheet="0" activeTab="0" autoFilterDateGrouping="1"/>
   </bookViews>
   <sheets>
-    <sheet name="Planilha 1" sheetId="1" state="visible" r:id="rId1"/>
+    <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Planilha 1" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames/>
   <calcPr calcId="0" fullCalcOnLoad="1" iterateDelta="0.0001"/>
@@ -694,7 +694,7 @@
       <c r="Y5" s="4" t="n"/>
       <c r="Z5" s="4" t="n"/>
     </row>
-    <row r="6" ht="84" customHeight="1">
+    <row r="6" ht="60" customHeight="1">
       <c r="A6" s="8" t="n">
         <v>1</v>
       </c>
@@ -710,14 +710,12 @@
       </c>
       <c r="D6" s="19" t="inlineStr">
         <is>
-          <t>1) Triagem Rápida: ao tocar em “Ver resultado” sem preencher todos os campos, o sistema não avisa nem indica o que falta, e não há retorno visual durante o cálculo (Severidade: Grande).
-2) Painel Meus Benefícios: a barra de progresso mostra o percentual, mas não informa quais etapas ou documentos faltam (Grande).
-3) Unidades: na busca por CEP não há indicador de carregamento; a tela parece travada durante a consulta (Grande).</t>
+          <t>As validações exibem alertas nativos do navegador (alert()) em vez de mensagem no próprio campo, em cadastro, triagem, simulação e adição de membro. O retorno interrompe o fluxo de forma abrupta (Severidade: Pequeno).</t>
         </is>
       </c>
       <c r="E6" s="19" t="inlineStr">
         <is>
-          <t>Sinalizar os campos obrigatórios e exibir indicador de carregamento na triagem; detalhar as pendências junto ao percentual do painel; mostrar indicador de carregamento durante a busca por CEP.</t>
+          <t>Substituir os alertas nativos por mensagens de estado e validação inline, junto ao campo correspondente.</t>
         </is>
       </c>
       <c r="F6" s="11" t="n"/>
@@ -742,7 +740,7 @@
       <c r="Y6" s="11" t="n"/>
       <c r="Z6" s="11" t="n"/>
     </row>
-    <row r="7" ht="66" customHeight="1">
+    <row r="7" ht="60" customHeight="1">
       <c r="A7" s="8" t="n">
         <v>2</v>
       </c>
@@ -758,13 +756,12 @@
       </c>
       <c r="D7" s="19" t="inlineStr">
         <is>
-          <t>1) Adicionar Membro: os campos “Parentesco” e “Vínculo” têm nomes parecidos e não explicam a diferença, confundindo o usuário (Pequeno).
-2) Resultado de elegibilidade: termos como “renda per capita”, “BPC” e “requisitos de elegibilidade” aparecem sem explicação acessível ao público-alvo (Grande).</t>
+          <t>Uso de vocabulário técnico e jurídico sem explicação ao público leigo: “elegibilidade”, “renda per capita”, “dossiê”, “CadÚnico”, “BPC” e “indeterminado”. Contraria a proposta de linguagem simples, RNF05 (Grande).</t>
         </is>
       </c>
       <c r="E7" s="19" t="inlineStr">
         <is>
-          <t>Usar rótulos em linguagem simples, com exemplos (ex.: Parentesco: filho, cônjuge); adicionar explicações curtas em linguagem simples junto de cada termo técnico.</t>
+          <t>Traduzir os termos para linguagem simples e acrescentar explicações curtas, acessíveis por toque, junto de cada ocorrência.</t>
         </is>
       </c>
       <c r="F7" s="11" t="n"/>
@@ -805,12 +802,12 @@
       </c>
       <c r="D8" s="19" t="inlineStr">
         <is>
-          <t>Perfil Familiar: a remoção de um membro ocorre imediatamente, sem confirmação nem opção de desfazer; um toque acidental apaga dados de renda já inseridos (Catastrófico).</t>
+          <t>Nenhum problema relevante identificado nesta heurística.</t>
         </is>
       </c>
       <c r="E8" s="19" t="inlineStr">
         <is>
-          <t>Exibir diálogo de confirmação antes de remover e oferecer opção de desfazer logo após a ação.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F8" s="11" t="n"/>
@@ -852,12 +849,12 @@
       </c>
       <c r="D9" s="19" t="inlineStr">
         <is>
-          <t>Navegação: o retorno à tela anterior aparece de duas formas (botão no topo e link no rodapé “Voltar para Perfil Familiar”), com posição variando entre telas (Cosmético).</t>
+          <t>O Painel do Colaborador exibia “Ola, [nome]!” e “Acesso rapido” sem acentuação, fora do padrão de escrita do app (Cosmético). Problema corrigido durante a avaliação.</t>
         </is>
       </c>
       <c r="E9" s="19" t="inlineStr">
         <is>
-          <t>Padronizar um único mecanismo de retorno, na mesma posição em todas as telas.</t>
+          <t>Padronizar a acentuação correta (“Olá”, “Acesso rápido”). Correção já aplicada.</t>
         </is>
       </c>
       <c r="F9" s="11" t="n"/>
@@ -882,7 +879,7 @@
       <c r="Y9" s="11" t="n"/>
       <c r="Z9" s="11" t="n"/>
     </row>
-    <row r="10" ht="84" customHeight="1">
+    <row r="10" ht="60" customHeight="1">
       <c r="A10" s="8" t="n">
         <v>5</v>
       </c>
@@ -898,14 +895,12 @@
       </c>
       <c r="D10" s="19" t="inlineStr">
         <is>
-          <t>1) Cadastro: o campo CPF só acusa formato inválido após o envio, com mensagem genérica (Grande).
-2) Simulação: o campo “Renda mensal total (R$)” aceita texto livre, sem máscara, gerando resultados inconsistentes (Grande).
-3) Cadastro: os campos de senha não informam os requisitos mínimos, e o erro só aparece depois do envio (Pequeno).</t>
+          <t>Nenhum problema relevante identificado nesta heurística.</t>
         </is>
       </c>
       <c r="E10" s="19" t="inlineStr">
         <is>
-          <t>Aplicar máscara e validação em tempo real no CPF; aplicar máscara de moeda e restringir a entrada a números no campo de renda; exibir os requisitos de senha antes do preenchimento.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F10" s="11" t="n"/>
@@ -946,12 +941,12 @@
       </c>
       <c r="D11" s="19" t="inlineStr">
         <is>
-          <t>Cadastro: os requisitos de senha (tamanho, caracteres) não são exibidos, exigindo que o usuário os memorize ou descubra por tentativa e erro (Pequeno).</t>
+          <t>Nenhum problema relevante identificado nesta heurística.</t>
         </is>
       </c>
       <c r="E11" s="19" t="inlineStr">
         <is>
-          <t>Exibir os requisitos sob o campo e um indicador de força que atualiza durante a digitação.</t>
+          <t>-</t>
         </is>
       </c>
       <c r="F11" s="11" t="n"/>
@@ -976,7 +971,7 @@
       <c r="Y11" s="11" t="n"/>
       <c r="Z11" s="11" t="n"/>
     </row>
-    <row r="12" ht="60" customHeight="1">
+    <row r="12" ht="70" customHeight="1">
       <c r="A12" s="8" t="n">
         <v>7</v>
       </c>
@@ -992,12 +987,13 @@
       </c>
       <c r="D12" s="19" t="inlineStr">
         <is>
-          <t>Nenhum problema relevante identificado nesta heurística.</t>
+          <t>1) Triagem (visitante) e Quiz (cadastrado) repetem as mesmas perguntas; as respostas da triagem não são reaproveitadas após o cadastro, gerando retrabalho (Pequeno).
+2) Após criar a conta, o usuário é levado de volta ao login e precisa autenticar de novo, em vez de já entrar autenticado (Pequeno).</t>
         </is>
       </c>
       <c r="E12" s="19" t="inlineStr">
         <is>
-          <t>-</t>
+          <t>Reaproveitar as respostas da triagem ao concluir o cadastro (ou unificar os fluxos) e autenticar o usuário automaticamente logo após o cadastro.</t>
         </is>
       </c>
       <c r="F12" s="11" t="n"/>
@@ -1068,7 +1064,7 @@
       <c r="Y13" s="11" t="n"/>
       <c r="Z13" s="11" t="n"/>
     </row>
-    <row r="14" ht="66" customHeight="1">
+    <row r="14" ht="60" customHeight="1">
       <c r="A14" s="8" t="n">
         <v>9</v>
       </c>
@@ -1084,13 +1080,12 @@
       </c>
       <c r="D14" s="19" t="inlineStr">
         <is>
-          <t>1) Cadastro: a mensagem de erro do CPF é genérica e não orienta a correção (Grande).
-2) Unidades: CEPs inexistentes não geram mensagem clara de erro (Grande).</t>
+          <t>As mensagens de erro aparecem em alert() genérico, sem orientar a correção no próprio campo (Pequeno).</t>
         </is>
       </c>
       <c r="E14" s="19" t="inlineStr">
         <is>
-          <t>Apresentar mensagens específicas que indiquem o que corrigir, tanto no CPF quanto na busca por CEP inválido ou não encontrado.</t>
+          <t>Apresentar mensagens específicas inline que indiquem o que corrigir, próximas ao campo com erro.</t>
         </is>
       </c>
       <c r="F14" s="11" t="n"/>
@@ -1131,7 +1126,7 @@
       </c>
       <c r="D15" s="21" t="inlineStr">
         <is>
-          <t>Resultado e detalhe do benefício: ausência de ajuda contextual para termos técnicos e para o significado dos requisitos de cada benefício (Grande).</t>
+          <t>Os termos técnicos da interface não têm ajuda contextual que explique seu significado ao usuário (Grande).</t>
         </is>
       </c>
       <c r="E15" s="21" t="inlineStr">

</xml_diff>